<commit_message>
Live streaming intake + rename demo client to Atlas Components Group
Ships the previously uncommitted live-intake experience (empty start,
drag-and-drop analysis streamed by narration.py, 33-test suite) and
renames the synthetic demo client Aurora Global Group -> Atlas
Components Group so one client threads through the full demo suite
(SEC screener -> tax-impact -> this copilot). Story tab reframes the
engagement as Atlas's six-jurisdiction first-wave GIR readiness pilot.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sample_inputs/trial_balance_by_entity.xlsx
+++ b/data/sample_inputs/trial_balance_by_entity.xlsx
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Aurora US, Inc.</t>
+          <t>Atlas US, Inc.</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -477,7 +477,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Aurora IE Holdings Ltd</t>
+          <t>Atlas IE Holdings Ltd</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -496,7 +496,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aurora DE GmbH</t>
+          <t>Atlas DE GmbH</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -515,7 +515,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Aurora NL BV</t>
+          <t>Atlas NL BV</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -532,7 +532,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Aurora SG IP Pte. Ltd</t>
+          <t>Atlas SG IP Pte. Ltd</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -549,7 +549,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Aurora UK Service Ltd</t>
+          <t>Atlas UK Service Ltd</t>
         </is>
       </c>
       <c r="B7" t="n">

</xml_diff>